<commit_message>
Location: Fredericton, NB; rebuild BOM and project book
</commit_message>
<xml_diff>
--- a/bom/Filament_Falcon_BOM.xlsx
+++ b/bom/Filament_Falcon_BOM.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="564">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -863,7 +863,7 @@
     <t xml:space="preserve">2x4 SPF stud 8 ft (2438 mm), kiln dried</t>
   </si>
   <si>
-    <t xml:space="preserve">22 used by the cut list + 2 spares. 38 x 89 mm (1.5" x 3.5"). Pick straight boards. Kent web price (store shown: Edmundston) - Moncton may differ</t>
+    <t xml:space="preserve">22 used by the cut list + 2 spares. 38 x 89 mm (1.5" x 3.5"). Pick straight boards. Kent Fredericton price (South/Bishop Dr and North/Two Nations Crossing, same price) checked 2026-10-09</t>
   </si>
   <si>
     <t xml:space="preserve">Frame (see frame/cut_list.md)</t>
@@ -878,19 +878,22 @@
     <t xml:space="preserve">https://kent.ca/en/search?q=2x4x8+stud</t>
   </si>
   <si>
-    <t xml:space="preserve">Kent.ca web price (Edmundston store shown)</t>
+    <t xml:space="preserve">2026-10-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kent.ca web price (Fredericton store)</t>
   </si>
   <si>
     <t xml:space="preserve">2x4 SPF 10 ft (3048 mm), kiln dried</t>
   </si>
   <si>
-    <t xml:space="preserve">The two 2450 mm sills. Kent web price from category listing</t>
+    <t xml:space="preserve">The two 2450 mm sills. Kent Fredericton price checked 2026-10-09</t>
   </si>
   <si>
     <t xml:space="preserve">Base sills</t>
   </si>
   <si>
-    <t xml:space="preserve">https://kent.ca/en/shop/building-materials/lumber-plywood/dimensional-lumber-studs</t>
+    <t xml:space="preserve">https://kent.ca/en/2-x-4-x-10-2-better-spf-lumber-kiln-dried-1016338</t>
   </si>
   <si>
     <t xml:space="preserve">https://kent.ca/en/search?q=2x4x10</t>
@@ -1106,7 +1109,7 @@
     <t xml:space="preserve">Local metal supplier</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.google.com/search?q=25mm+steel+round+bar+Moncton+NB</t>
+    <t xml:space="preserve">https://www.google.com/search?q=25mm+steel+round+bar+Fredericton+NB</t>
   </si>
   <si>
     <t xml:space="preserve">Estimate - get a quote</t>
@@ -1172,7 +1175,7 @@
     <t xml:space="preserve">Under the pod bearings / supports on the tower posts. Metal shop or cut from flat bar</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.google.com/search?q=6mm+steel+plate+Moncton+NB</t>
+    <t xml:space="preserve">https://www.google.com/search?q=6mm+steel+plate+Fredericton+NB</t>
   </si>
   <si>
     <t xml:space="preserve">M10 x 90 coach screws + washers</t>
@@ -1283,7 +1286,7 @@
     <t xml:space="preserve">Pod mechanical locks</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.google.com/search?q=laser+cutting+steel+plate+moncton+Moncton+NB</t>
+    <t xml:space="preserve">https://www.google.com/search?q=laser+cutting+steel+plate+Fredericton+NB</t>
   </si>
   <si>
     <t xml:space="preserve">Spring-loaded steel pawl (barrel bolt / gate latch)</t>
@@ -1718,7 +1721,7 @@
     <t xml:space="preserve">Amazon cart total</t>
   </si>
   <si>
-    <t xml:space="preserve">The Filament Falcon - BOM notes (built 2026-10-08, America/Moncton)</t>
+    <t xml:space="preserve">The Filament Falcon - BOM notes (built 2026-10-09, Atlantic time ADT/AST; location Fredericton, NB)</t>
   </si>
   <si>
     <t xml:space="preserve">Sources: filament-falcon/docs/SPEC.md; ff-fw/docs/electronics/README.md; ff-cad (branch cad, commit b743d58): frame/BOM.md v0.2, frame/cut_list.md, docs/mechanical/README.md, switch_bom.md, displays.md.</t>
@@ -1730,7 +1733,7 @@
     <t xml:space="preserve">Filament result: black 3601 cm3 -&gt; 5.26 kg (buy 6 x 1 kg); white 44 cm3 -&gt; 0.06 kg (buy 1 x 1 kg). Red/grey parts (guard lids, throttle grip, gear arm, adapter plates) are counted in black - print them in red/grey if you have it. PLA would need ~2 % less mass, but PETG is required for the harness hub and recommended everywhere.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prices: "Verified amazon.ca price" = read from the amazon.ca product page on 2026-10-08 (buy-box price, CAD, before tax). Kent prices are from kent.ca (store shown online: Edmundston); Moncton store prices may differ. Rows marked Estimate/placeholder are NOT verified prices.</t>
+    <t xml:space="preserve">Prices: "Verified amazon.ca price" = read from the amazon.ca product page on 2026-10-08 (buy-box price, CAD, before tax). Kent prices were read from kent.ca on 2026-10-09 with the Fredericton store selected (Fredericton South, 809 Bishop Dr, and Fredericton North, 25 Two Nations Crossing showed identical prices); they can change, check before buying. Local metal-supplier rows have Google search links for Fredericton NB. Rows marked Estimate/placeholder are NOT verified prices.</t>
   </si>
   <si>
     <t xml:space="preserve">Motion system (v0.2, final per commit b743d58): 2 cradle actuators 10"/1500 N (~364 mm retracted), 2 pod actuators 12"/1000 N (~415 mm retracted), both self-locking; 2 gas struts ~590 N; 25 mm shafts, UCP205/UCF205/SHF25; spring pawls + latch plates + Bowden release; steel hard stops; key, E-stop, 20 A fuse, hold-to-run DPDT, relays as H-bridges, 10 roller limit switches, safety edge. Check actuator retracted length and self-locking before ordering.</t>
@@ -4869,7 +4872,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
         <v>267</v>
       </c>
@@ -4910,10 +4913,10 @@
         <v>273</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>42</v>
+        <v>274</v>
       </c>
       <c r="N53" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O53" s="6" t="str">
         <f aca="false">IF(AND(J53="Amazon.ca",G53&gt;0,ISERROR(SEARCH("ALTERNATIVE",A53))),MAX(O$1:O52)+1,"")</f>
@@ -4925,13 +4928,13 @@
         <v>267</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>2</v>
@@ -4955,16 +4958,16 @@
         <v>271</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L54" s="7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>42</v>
+        <v>274</v>
       </c>
       <c r="N54" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O54" s="6" t="str">
         <f aca="false">IF(AND(J54="Amazon.ca",G54&gt;0,ISERROR(SEARCH("ALTERNATIVE",A54))),MAX(O$1:O53)+1,"")</f>
@@ -4976,13 +4979,13 @@
         <v>267</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>6</v>
@@ -4996,26 +4999,26 @@
         <v>6</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>64.98</v>
+        <v>63.98</v>
       </c>
       <c r="I55" s="5" t="n">
         <f aca="false">IF(H55="","",G55*H55)</f>
-        <v>389.88</v>
+        <v>383.88</v>
       </c>
       <c r="J55" s="2" t="s">
         <v>271</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L55" s="7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>42</v>
+        <v>274</v>
       </c>
       <c r="N55" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O55" s="6" t="str">
         <f aca="false">IF(AND(J55="Amazon.ca",G55&gt;0,ISERROR(SEARCH("ALTERNATIVE",A55))),MAX(O$1:O54)+1,"")</f>
@@ -5027,13 +5030,13 @@
         <v>267</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>4</v>
@@ -5057,16 +5060,16 @@
         <v>271</v>
       </c>
       <c r="K56" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L56" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>42</v>
+        <v>274</v>
       </c>
       <c r="N56" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O56" s="6" t="str">
         <f aca="false">IF(AND(J56="Amazon.ca",G56&gt;0,ISERROR(SEARCH("ALTERNATIVE",A56))),MAX(O$1:O55)+1,"")</f>
@@ -5078,13 +5081,13 @@
         <v>267</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>1</v>
@@ -5108,16 +5111,16 @@
         <v>271</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L57" s="7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>42</v>
+        <v>274</v>
       </c>
       <c r="N57" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O57" s="6" t="str">
         <f aca="false">IF(AND(J57="Amazon.ca",G57&gt;0,ISERROR(SEARCH("ALTERNATIVE",A57))),MAX(O$1:O56)+1,"")</f>
@@ -5126,16 +5129,16 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1</v>
@@ -5156,15 +5159,15 @@
         <v>25</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K58" s="2"/>
       <c r="L58" s="7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="M58" s="2"/>
       <c r="N58" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O58" s="6" t="str">
         <f aca="false">IF(AND(J58="Amazon.ca",G58&gt;0,ISERROR(SEARCH("ALTERNATIVE",A58))),MAX(O$1:O57)+1,"")</f>
@@ -5173,16 +5176,16 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>1</v>
@@ -5203,15 +5206,15 @@
         <v>15</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K59" s="2"/>
       <c r="L59" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="M59" s="2"/>
       <c r="N59" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O59" s="6" t="str">
         <f aca="false">IF(AND(J59="Amazon.ca",G59&gt;0,ISERROR(SEARCH("ALTERNATIVE",A59))),MAX(O$1:O58)+1,"")</f>
@@ -5220,16 +5223,16 @@
     </row>
     <row r="60" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>1</v>
@@ -5250,15 +5253,15 @@
         <v>12</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K60" s="2"/>
       <c r="L60" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="M60" s="2"/>
       <c r="N60" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O60" s="6" t="str">
         <f aca="false">IF(AND(J60="Amazon.ca",G60&gt;0,ISERROR(SEARCH("ALTERNATIVE",A60))),MAX(O$1:O59)+1,"")</f>
@@ -5267,16 +5270,16 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>1</v>
@@ -5297,15 +5300,15 @@
         <v>15</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K61" s="2"/>
       <c r="L61" s="7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="M61" s="2"/>
       <c r="N61" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O61" s="6" t="str">
         <f aca="false">IF(AND(J61="Amazon.ca",G61&gt;0,ISERROR(SEARCH("ALTERNATIVE",A61))),MAX(O$1:O60)+1,"")</f>
@@ -5314,16 +5317,16 @@
     </row>
     <row r="62" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>1</v>
@@ -5347,10 +5350,10 @@
         <v>39</v>
       </c>
       <c r="K62" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="L62" s="7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="M62" s="2" t="s">
         <v>42</v>
@@ -5365,16 +5368,16 @@
     </row>
     <row r="63" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>4</v>
@@ -5398,10 +5401,10 @@
         <v>39</v>
       </c>
       <c r="K63" s="7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="L63" s="7" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M63" s="2" t="s">
         <v>42</v>
@@ -5416,16 +5419,16 @@
     </row>
     <row r="64" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>1</v>
@@ -5449,10 +5452,10 @@
         <v>39</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L64" s="7" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M64" s="2" t="s">
         <v>42</v>
@@ -5467,16 +5470,16 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>8</v>
@@ -5497,15 +5500,15 @@
         <v>12</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K65" s="2"/>
       <c r="L65" s="7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="M65" s="2"/>
       <c r="N65" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O65" s="6" t="str">
         <f aca="false">IF(AND(J65="Amazon.ca",G65&gt;0,ISERROR(SEARCH("ALTERNATIVE",A65))),MAX(O$1:O64)+1,"")</f>
@@ -5514,16 +5517,16 @@
     </row>
     <row r="66" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>1</v>
@@ -5547,10 +5550,10 @@
         <v>39</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="L66" s="7" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="M66" s="2" t="s">
         <v>42</v>
@@ -5565,16 +5568,16 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>1</v>
@@ -5595,15 +5598,15 @@
         <v>4</v>
       </c>
       <c r="J67" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K67" s="2"/>
       <c r="L67" s="7" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="M67" s="2"/>
       <c r="N67" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O67" s="6" t="str">
         <f aca="false">IF(AND(J67="Amazon.ca",G67&gt;0,ISERROR(SEARCH("ALTERNATIVE",A67))),MAX(O$1:O66)+1,"")</f>
@@ -5612,16 +5615,16 @@
     </row>
     <row r="68" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>1</v>
@@ -5645,10 +5648,10 @@
         <v>39</v>
       </c>
       <c r="K68" s="7" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="L68" s="7" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="M68" s="2" t="s">
         <v>42</v>
@@ -5663,16 +5666,16 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>1</v>
@@ -5693,15 +5696,15 @@
         <v>30</v>
       </c>
       <c r="J69" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K69" s="2"/>
       <c r="L69" s="7" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M69" s="2"/>
       <c r="N69" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="O69" s="6" t="str">
         <f aca="false">IF(AND(J69="Amazon.ca",G69&gt;0,ISERROR(SEARCH("ALTERNATIVE",A69))),MAX(O$1:O68)+1,"")</f>
@@ -5710,16 +5713,16 @@
     </row>
     <row r="70" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>2</v>
@@ -5743,10 +5746,10 @@
         <v>39</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="L70" s="7" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="M70" s="2" t="s">
         <v>42</v>
@@ -5761,16 +5764,16 @@
     </row>
     <row r="71" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>1</v>
@@ -5794,10 +5797,10 @@
         <v>39</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="L71" s="7" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="M71" s="2" t="s">
         <v>42</v>
@@ -5812,16 +5815,16 @@
     </row>
     <row r="72" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>2</v>
@@ -5845,10 +5848,10 @@
         <v>39</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="L72" s="7" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="M72" s="2" t="s">
         <v>42</v>
@@ -5863,16 +5866,16 @@
     </row>
     <row r="73" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>2</v>
@@ -5896,10 +5899,10 @@
         <v>39</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="L73" s="7" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="M73" s="2" t="s">
         <v>42</v>
@@ -5914,16 +5917,16 @@
     </row>
     <row r="74" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>4</v>
@@ -5944,15 +5947,15 @@
         <v>40</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K74" s="2"/>
       <c r="L74" s="7" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="M74" s="2"/>
       <c r="N74" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="O74" s="6" t="str">
         <f aca="false">IF(AND(J74="Amazon.ca",G74&gt;0,ISERROR(SEARCH("ALTERNATIVE",A74))),MAX(O$1:O73)+1,"")</f>
@@ -5961,16 +5964,16 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>20</v>
@@ -5991,15 +5994,15 @@
         <v>25</v>
       </c>
       <c r="J75" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K75" s="2"/>
       <c r="L75" s="7" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M75" s="2"/>
       <c r="N75" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O75" s="6" t="str">
         <f aca="false">IF(AND(J75="Amazon.ca",G75&gt;0,ISERROR(SEARCH("ALTERNATIVE",A75))),MAX(O$1:O74)+1,"")</f>
@@ -6008,16 +6011,16 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>8</v>
@@ -6038,15 +6041,15 @@
         <v>12</v>
       </c>
       <c r="J76" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K76" s="2"/>
       <c r="L76" s="7" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M76" s="2"/>
       <c r="N76" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O76" s="6" t="str">
         <f aca="false">IF(AND(J76="Amazon.ca",G76&gt;0,ISERROR(SEARCH("ALTERNATIVE",A76))),MAX(O$1:O75)+1,"")</f>
@@ -6055,16 +6058,16 @@
     </row>
     <row r="77" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>2</v>
@@ -6088,10 +6091,10 @@
         <v>39</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="L77" s="7" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="M77" s="2" t="s">
         <v>42</v>
@@ -6106,16 +6109,16 @@
     </row>
     <row r="78" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>2</v>
@@ -6139,10 +6142,10 @@
         <v>39</v>
       </c>
       <c r="K78" s="7" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="L78" s="7" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="M78" s="2" t="s">
         <v>42</v>
@@ -6157,16 +6160,16 @@
     </row>
     <row r="79" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>1</v>
@@ -6190,10 +6193,10 @@
         <v>39</v>
       </c>
       <c r="K79" s="7" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="L79" s="7" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="M79" s="2" t="s">
         <v>42</v>
@@ -6208,16 +6211,16 @@
     </row>
     <row r="80" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>1</v>
@@ -6241,10 +6244,10 @@
         <v>39</v>
       </c>
       <c r="K80" s="7" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L80" s="7" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M80" s="2" t="s">
         <v>42</v>
@@ -6259,16 +6262,16 @@
     </row>
     <row r="81" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>4</v>
@@ -6289,15 +6292,15 @@
         <v>32</v>
       </c>
       <c r="J81" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K81" s="2"/>
       <c r="L81" s="7" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="M81" s="2"/>
       <c r="N81" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O81" s="6" t="str">
         <f aca="false">IF(AND(J81="Amazon.ca",G81&gt;0,ISERROR(SEARCH("ALTERNATIVE",A81))),MAX(O$1:O80)+1,"")</f>
@@ -6306,16 +6309,16 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>2</v>
@@ -6336,15 +6339,15 @@
         <v>50</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K82" s="2"/>
       <c r="L82" s="7" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M82" s="2"/>
       <c r="N82" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="O82" s="6" t="str">
         <f aca="false">IF(AND(J82="Amazon.ca",G82&gt;0,ISERROR(SEARCH("ALTERNATIVE",A82))),MAX(O$1:O81)+1,"")</f>
@@ -6353,16 +6356,16 @@
     </row>
     <row r="83" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>2</v>
@@ -6386,10 +6389,10 @@
         <v>39</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="L83" s="7" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="M83" s="2" t="s">
         <v>42</v>
@@ -6404,16 +6407,16 @@
     </row>
     <row r="84" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>1</v>
@@ -6437,10 +6440,10 @@
         <v>39</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="L84" s="7" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="M84" s="2" t="s">
         <v>42</v>
@@ -6455,16 +6458,16 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>4</v>
@@ -6485,15 +6488,15 @@
         <v>16</v>
       </c>
       <c r="J85" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K85" s="2"/>
       <c r="L85" s="7" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="M85" s="2"/>
       <c r="N85" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O85" s="6" t="str">
         <f aca="false">IF(AND(J85="Amazon.ca",G85&gt;0,ISERROR(SEARCH("ALTERNATIVE",A85))),MAX(O$1:O84)+1,"")</f>
@@ -6502,16 +6505,16 @@
     </row>
     <row r="86" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>1</v>
@@ -6535,10 +6538,10 @@
         <v>39</v>
       </c>
       <c r="K86" s="7" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="L86" s="7" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M86" s="2" t="s">
         <v>42</v>
@@ -6553,16 +6556,16 @@
     </row>
     <row r="87" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>1</v>
@@ -6586,10 +6589,10 @@
         <v>39</v>
       </c>
       <c r="K87" s="7" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="L87" s="7" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M87" s="2" t="s">
         <v>42</v>
@@ -6604,16 +6607,16 @@
     </row>
     <row r="88" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>1</v>
@@ -6637,10 +6640,10 @@
         <v>39</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="L88" s="7" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="M88" s="2" t="s">
         <v>42</v>
@@ -6655,16 +6658,16 @@
     </row>
     <row r="89" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>1</v>
@@ -6706,16 +6709,16 @@
     </row>
     <row r="90" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>1</v>
@@ -6739,10 +6742,10 @@
         <v>39</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L90" s="7" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="M90" s="2" t="s">
         <v>42</v>
@@ -6757,16 +6760,16 @@
     </row>
     <row r="91" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>1</v>
@@ -6790,10 +6793,10 @@
         <v>39</v>
       </c>
       <c r="K91" s="7" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="L91" s="7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="M91" s="2" t="s">
         <v>42</v>
@@ -6808,16 +6811,16 @@
     </row>
     <row r="92" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>1</v>
@@ -6841,10 +6844,10 @@
         <v>39</v>
       </c>
       <c r="K92" s="7" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="L92" s="7" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="M92" s="2" t="s">
         <v>42</v>
@@ -6859,16 +6862,16 @@
     </row>
     <row r="93" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>2</v>
@@ -6892,10 +6895,10 @@
         <v>39</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="L93" s="7" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M93" s="2" t="s">
         <v>42</v>
@@ -6910,16 +6913,16 @@
     </row>
     <row r="94" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>1</v>
@@ -6943,10 +6946,10 @@
         <v>39</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L94" s="7" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="M94" s="2" t="s">
         <v>42</v>
@@ -6961,16 +6964,16 @@
     </row>
     <row r="95" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>1</v>
@@ -6991,15 +6994,15 @@
         <v>150</v>
       </c>
       <c r="J95" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K95" s="2"/>
       <c r="L95" s="7" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="M95" s="2"/>
       <c r="N95" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="O95" s="6" t="str">
         <f aca="false">IF(AND(J95="Amazon.ca",G95&gt;0,ISERROR(SEARCH("ALTERNATIVE",A95))),MAX(O$1:O94)+1,"")</f>
@@ -7008,16 +7011,16 @@
     </row>
     <row r="96" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>2</v>
@@ -7041,10 +7044,10 @@
         <v>39</v>
       </c>
       <c r="K96" s="7" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="L96" s="7" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="M96" s="2" t="s">
         <v>42</v>
@@ -7059,16 +7062,16 @@
     </row>
     <row r="97" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>1</v>
@@ -7092,10 +7095,10 @@
         <v>39</v>
       </c>
       <c r="K97" s="7" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="L97" s="7" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M97" s="2" t="s">
         <v>42</v>
@@ -7110,16 +7113,16 @@
     </row>
     <row r="98" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>1</v>
@@ -7144,7 +7147,7 @@
       </c>
       <c r="K98" s="2"/>
       <c r="L98" s="7" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="M98" s="2"/>
       <c r="N98" s="3" t="s">
@@ -7157,16 +7160,16 @@
     </row>
     <row r="99" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E99" s="2" t="n">
         <v>1</v>
@@ -7190,10 +7193,10 @@
         <v>39</v>
       </c>
       <c r="K99" s="7" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="L99" s="7" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="M99" s="2" t="s">
         <v>42</v>
@@ -7208,16 +7211,16 @@
     </row>
     <row r="100" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>1</v>
@@ -7241,16 +7244,16 @@
         <v>39</v>
       </c>
       <c r="K100" s="7" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="L100" s="7" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="M100" s="2" t="s">
         <v>42</v>
       </c>
       <c r="N100" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="O100" s="6" t="n">
         <f aca="false">IF(AND(J100="Amazon.ca",G100&gt;0,ISERROR(SEARCH("ALTERNATIVE",A100))),MAX(O$1:O99)+1,"")</f>
@@ -7259,16 +7262,16 @@
     </row>
     <row r="101" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>1</v>
@@ -7292,10 +7295,10 @@
         <v>39</v>
       </c>
       <c r="K101" s="7" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="L101" s="7" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="M101" s="2" t="s">
         <v>42</v>
@@ -7310,16 +7313,16 @@
     </row>
     <row r="102" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>1</v>
@@ -7343,10 +7346,10 @@
         <v>39</v>
       </c>
       <c r="K102" s="7" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="L102" s="7" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="M102" s="2" t="s">
         <v>42</v>
@@ -7361,16 +7364,16 @@
     </row>
     <row r="103" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>1</v>
@@ -7394,10 +7397,10 @@
         <v>39</v>
       </c>
       <c r="K103" s="7" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="L103" s="7" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="M103" s="2" t="s">
         <v>42</v>
@@ -7412,16 +7415,16 @@
     </row>
     <row r="104" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>10</v>
@@ -7442,15 +7445,15 @@
         <v>60</v>
       </c>
       <c r="J104" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K104" s="2"/>
       <c r="L104" s="7" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="M104" s="2"/>
       <c r="N104" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O104" s="6" t="str">
         <f aca="false">IF(AND(J104="Amazon.ca",G104&gt;0,ISERROR(SEARCH("ALTERNATIVE",A104))),MAX(O$1:O103)+1,"")</f>
@@ -7459,16 +7462,16 @@
     </row>
     <row r="105" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>1</v>
@@ -7492,10 +7495,10 @@
         <v>39</v>
       </c>
       <c r="K105" s="7" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="L105" s="7" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="M105" s="2" t="s">
         <v>42</v>
@@ -7510,16 +7513,16 @@
     </row>
     <row r="106" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>1</v>
@@ -7543,10 +7546,10 @@
         <v>39</v>
       </c>
       <c r="K106" s="7" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="L106" s="7" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="M106" s="2" t="s">
         <v>42</v>
@@ -7561,16 +7564,16 @@
     </row>
     <row r="107" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>1</v>
@@ -7594,10 +7597,10 @@
         <v>39</v>
       </c>
       <c r="K107" s="7" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="L107" s="7" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="M107" s="2" t="s">
         <v>42</v>
@@ -7612,16 +7615,16 @@
     </row>
     <row r="108" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>2</v>
@@ -7645,10 +7648,10 @@
         <v>39</v>
       </c>
       <c r="K108" s="7" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="L108" s="7" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="M108" s="2" t="s">
         <v>42</v>
@@ -7769,7 +7772,7 @@
     <hyperlink ref="L52" r:id="rId89" display="https://www.amazon.ca/s?k=self+tapping+screw+assortment+m2.5+m3"/>
     <hyperlink ref="K53" r:id="rId90" display="https://kent.ca/en/2-x-4-x-8-spf-stud-kiln-dried-1016318"/>
     <hyperlink ref="L53" r:id="rId91" display="https://kent.ca/en/search?q=2x4x8+stud"/>
-    <hyperlink ref="K54" r:id="rId92" display="https://kent.ca/en/shop/building-materials/lumber-plywood/dimensional-lumber-studs"/>
+    <hyperlink ref="K54" r:id="rId92" display="https://kent.ca/en/2-x-4-x-10-2-better-spf-lumber-kiln-dried-1016338"/>
     <hyperlink ref="L54" r:id="rId93" display="https://kent.ca/en/search?q=2x4x10"/>
     <hyperlink ref="K55" r:id="rId94" display="https://kent.ca/en/3-4-x-4-x-8-18-5mm-spruce-plywood-standard-1015824"/>
     <hyperlink ref="L55" r:id="rId95" display="https://kent.ca/en/search?q=3%2F4+plywood+4x8"/>
@@ -7793,7 +7796,7 @@
     <hyperlink ref="L67" r:id="rId113" display="https://kent.ca/en/search?q=m6+x+30+bolt"/>
     <hyperlink ref="K68" r:id="rId114" display="https://www.amazon.ca/dp/B0G5ZDQB47"/>
     <hyperlink ref="L68" r:id="rId115" display="https://www.amazon.ca/s?k=25mm+shaft+1000mm"/>
-    <hyperlink ref="L69" r:id="rId116" display="https://www.google.com/search?q=25mm+steel+round+bar+Moncton+NB"/>
+    <hyperlink ref="L69" r:id="rId116" display="https://www.google.com/search?q=25mm+steel+round+bar+Fredericton+NB"/>
     <hyperlink ref="K70" r:id="rId117" display="https://www.amazon.ca/dp/B0D9RTBQF2"/>
     <hyperlink ref="L70" r:id="rId118" display="https://www.amazon.ca/s?k=shf25+shaft+support"/>
     <hyperlink ref="K71" r:id="rId119" display="https://www.amazon.ca/dp/B08HJYZK1X"/>
@@ -7802,7 +7805,7 @@
     <hyperlink ref="L72" r:id="rId122" display="https://www.amazon.ca/s?k=ucf205+flange+bearing+25mm"/>
     <hyperlink ref="K73" r:id="rId123" display="https://www.amazon.ca/dp/B0G2Q98L26"/>
     <hyperlink ref="L73" r:id="rId124" display="https://www.amazon.ca/s?k=25mm+shaft+collar+steel"/>
-    <hyperlink ref="L74" r:id="rId125" display="https://www.google.com/search?q=6mm+steel+plate+Moncton+NB"/>
+    <hyperlink ref="L74" r:id="rId125" display="https://www.google.com/search?q=6mm+steel+plate+Fredericton+NB"/>
     <hyperlink ref="L75" r:id="rId126" display="https://kent.ca/en/search?q=m10+x+90+lag+screw"/>
     <hyperlink ref="L76" r:id="rId127" display="https://kent.ca/en/search?q=m8+x+60+bolt"/>
     <hyperlink ref="K77" r:id="rId128" display="https://www.amazon.ca/dp/B0FKMS7Y12"/>
@@ -7814,7 +7817,7 @@
     <hyperlink ref="K80" r:id="rId134" display="https://www.amazon.ca/dp/B07SJ6B3QP"/>
     <hyperlink ref="L80" r:id="rId135" display="https://www.amazon.ca/s?k=10mm+ball+stud+gas+strut+bracket"/>
     <hyperlink ref="L81" r:id="rId136" display="https://kent.ca/en/search?q=heavy+steel+angle+bracket"/>
-    <hyperlink ref="L82" r:id="rId137" display="https://www.google.com/search?q=laser+cutting+steel+plate+moncton+Moncton+NB"/>
+    <hyperlink ref="L82" r:id="rId137" display="https://www.google.com/search?q=laser+cutting+steel+plate+Fredericton+NB"/>
     <hyperlink ref="K83" r:id="rId138" display="https://www.amazon.ca/dp/B07GZHSCP6"/>
     <hyperlink ref="L83" r:id="rId139" display="https://www.amazon.ca/s?k=spring+loaded+barrel+bolt+latch+heavy+duty"/>
     <hyperlink ref="K84" r:id="rId140" display="https://www.amazon.ca/dp/B0B8C66T4Q"/>
@@ -7893,13 +7896,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8018,12 +8021,12 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">SUMIF(BOM!$A$2:$A$108,A8,BOM!$I$2:$I$108)</f>
-        <v>682.07</v>
+        <v>676.07</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">COUNTIF(BOM!$A$2:$A$108,A9)</f>
@@ -8040,7 +8043,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B10" s="0" t="n">
         <f aca="false">COUNTIF(BOM!$A$2:$A$108,A10)</f>
@@ -8057,7 +8060,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">COUNTIF(BOM!$A$2:$A$108,A11)</f>
@@ -8074,7 +8077,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">COUNTIF(BOM!$A$2:$A$108,A12)</f>
@@ -8091,7 +8094,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B13" s="0" t="n">
         <f aca="false">COUNTIF(BOM!$A$2:$A$108,A13)</f>
@@ -8108,7 +8111,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B14" s="0" t="n">
         <f aca="false">COUNTIF(BOM!$A$2:$A$108,A14)</f>
@@ -8125,7 +8128,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B15" s="0" t="n">
         <f aca="false">COUNTIF(BOM!$A$2:$A$108,A15)</f>
@@ -8142,7 +8145,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">SUMPRODUCT((ISERROR(SEARCH("ALTERNATIVE",A2:A15)))*C2:C15)</f>
@@ -8150,12 +8153,12 @@
       </c>
       <c r="D17" s="11" t="n">
         <f aca="false">SUMPRODUCT((ISERROR(SEARCH("ALTERNATIVE",A2:A15)))*D2:D15)</f>
-        <v>3370.04</v>
+        <v>3364.04</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">SUMPRODUCT((BOM!$J$2:$J$108="Amazon.ca")*ISERROR(SEARCH("ALTERNATIVE",BOM!$A$2:$A$108))*N(+BOM!$I$2:$I$108))</f>
@@ -8164,16 +8167,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">SUMPRODUCT(ISNUMBER(SEARCH("Kent",BOM!$J$2:$J$108))*N(+BOM!$I$2:$I$108))</f>
-        <v>910.07</v>
+        <v>904.07</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D20" s="9" t="n">
         <f aca="false">SUMPRODUCT((ISNUMBER(SEARCH("supplier",BOM!$J$2:$J$108)))*N(+BOM!$I$2:$I$108))</f>
@@ -8182,16 +8185,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">SUMPRODUCT((ISNUMBER(SEARCH("Verified amazon.ca price",BOM!$N$2:$N$108))+ISNUMBER(SEARCH("Kent.ca web price",BOM!$N$2:$N$108))&gt;0)*ISERROR(SEARCH("ALTERNATIVE",BOM!$A$2:$A$108))*N(+BOM!$I$2:$I$108))</f>
-        <v>2779.04</v>
+        <v>2773.04</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">SUMPRODUCT((ISNUMBER(SEARCH("estimate",BOM!$N$2:$N$108)))*ISERROR(SEARCH("ALTERNATIVE",BOM!$A$2:$A$108))*N(+BOM!$I$2:$I$108))</f>
@@ -8200,7 +8203,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUMPRODUCT(ISNUMBER(SEARCH("ALTERNATIVE",BOM!$A$2:$A$108))*N(+BOM!$I$2:$I$108))</f>
@@ -8209,12 +8212,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -8246,7 +8249,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>1</v>
@@ -8267,7 +8270,7 @@
         <v>11</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11872,7 +11875,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="10" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="E123" s="9" t="n">
         <f aca="false">SUM(E2:E121)</f>
@@ -11903,47 +11906,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>